<commit_message>
fixing up some ITRA data issues... about time! ha!
</commit_message>
<xml_diff>
--- a/TOR130 Data/5. Clean Data for Data Visualisation/TOR130_itra_including_DNF.xlsx
+++ b/TOR130 Data/5. Clean Data for Data Visualisation/TOR130_itra_including_DNF.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Name</t>
   </si>
@@ -41,6 +41,18 @@
   </si>
   <si>
     <t>Race</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Race </t>
+  </si>
+  <si>
+    <t>Race Age</t>
+  </si>
+  <si>
+    <t>Race Score</t>
+  </si>
+  <si>
+    <t>Status1</t>
   </si>
 </sst>
 </file>
@@ -398,10 +410,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -428,6 +440,18 @@
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>